<commit_message>
Add XmlWriter and wrapper classes for JAXB support
</commit_message>
<xml_diff>
--- a/src/main/resources/universityInfoStatistics.xlsx
+++ b/src/main/resources/universityInfoStatistics.xlsx
@@ -35,22 +35,22 @@
     <t>Казанский Университет Вычислений;</t>
   </si>
   <si>
+    <t>Физика</t>
+  </si>
+  <si>
+    <t>Московский Выдуманный Университет;Московский Придуманный Институт;</t>
+  </si>
+  <si>
+    <t>Лингвистика</t>
+  </si>
+  <si>
+    <t>Воронежский Литературно-Переводческий Университет;</t>
+  </si>
+  <si>
     <t>Медицина</t>
   </si>
   <si>
     <t>Московский Государственный Медицинский Университет;Тамбовский Университет Медицины;Самарский Медицинский Институт;</t>
-  </si>
-  <si>
-    <t>Лингвистика</t>
-  </si>
-  <si>
-    <t>Воронежский Литературно-Переводческий Университет;</t>
-  </si>
-  <si>
-    <t>Физика</t>
-  </si>
-  <si>
-    <t>Московский Выдуманный Университет;Московский Придуманный Институт;</t>
   </si>
 </sst>
 </file>
@@ -150,16 +150,16 @@
         <v>7</v>
       </c>
       <c r="B3" t="n" s="0">
-        <v>4.329999923706055</v>
+        <v>4.539999961853027</v>
       </c>
       <c r="C3" t="n" s="0">
-        <v>3.0</v>
+        <v>8.0</v>
       </c>
       <c r="D3" t="s" s="0">
         <v>8</v>
       </c>
       <c r="E3" t="n" s="0">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="4">
@@ -184,16 +184,16 @@
         <v>11</v>
       </c>
       <c r="B5" t="n" s="0">
-        <v>4.539999961853027</v>
+        <v>4.329999923706055</v>
       </c>
       <c r="C5" t="n" s="0">
-        <v>8.0</v>
+        <v>3.0</v>
       </c>
       <c r="D5" t="s" s="0">
         <v>12</v>
       </c>
       <c r="E5" t="n" s="0">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>